<commit_message>
Licence fee B$60,000; half-up rounding of escalated amounts
</commit_message>
<xml_diff>
--- a/docs/proposal/IIFT-Commercial-Pricing-iorta-TechNXT.xlsx
+++ b/docs/proposal/IIFT-Commercial-Pricing-iorta-TechNXT.xlsx
@@ -2421,10 +2421,10 @@
         </is>
       </c>
       <c r="D6" s="11" t="n">
-        <v>26000</v>
+        <v>32500</v>
       </c>
       <c r="E6" s="11" t="n">
-        <v>22000</v>
+        <v>27500</v>
       </c>
       <c r="F6" s="11">
         <f>D6+E6</f>
@@ -3204,10 +3204,10 @@
         </is>
       </c>
       <c r="D34" s="17" t="n">
-        <v>18365</v>
+        <v>19866</v>
       </c>
       <c r="E34" s="17" t="n">
-        <v>14553</v>
+        <v>15824</v>
       </c>
       <c r="F34" s="17">
         <f>D34+E34</f>
@@ -3240,10 +3240,10 @@
         </is>
       </c>
       <c r="D35" s="11" t="n">
-        <v>19283</v>
+        <v>20859</v>
       </c>
       <c r="E35" s="11" t="n">
-        <v>15281</v>
+        <v>16615</v>
       </c>
       <c r="F35" s="11">
         <f>D35+E35</f>
@@ -3276,10 +3276,10 @@
         </is>
       </c>
       <c r="D36" s="17" t="n">
-        <v>20247</v>
+        <v>21902</v>
       </c>
       <c r="E36" s="17" t="n">
-        <v>16045</v>
+        <v>17445</v>
       </c>
       <c r="F36" s="17">
         <f>D36+E36</f>
@@ -3312,10 +3312,10 @@
         </is>
       </c>
       <c r="D37" s="11" t="n">
-        <v>21259</v>
+        <v>22997</v>
       </c>
       <c r="E37" s="11" t="n">
-        <v>16847</v>
+        <v>18318</v>
       </c>
       <c r="F37" s="11">
         <f>D37+E37</f>
@@ -5652,7 +5652,7 @@
         </is>
       </c>
       <c r="D45" s="17" t="n">
-        <v>14963</v>
+        <v>16223</v>
       </c>
       <c r="E45" s="17">
         <f>'Option A'!$F$34</f>
@@ -5681,7 +5681,7 @@
         </is>
       </c>
       <c r="D46" s="11" t="n">
-        <v>15711</v>
+        <v>17034</v>
       </c>
       <c r="E46" s="11">
         <f>'Option A'!$F$35</f>
@@ -5710,7 +5710,7 @@
         </is>
       </c>
       <c r="D47" s="17" t="n">
-        <v>16496</v>
+        <v>17885</v>
       </c>
       <c r="E47" s="17">
         <f>'Option A'!$F$36</f>
@@ -5739,7 +5739,7 @@
         </is>
       </c>
       <c r="D48" s="11" t="n">
-        <v>17321</v>
+        <v>18780</v>
       </c>
       <c r="E48" s="11">
         <f>'Option A'!$F$37</f>
@@ -6014,10 +6014,10 @@
         </is>
       </c>
       <c r="D5" s="11" t="n">
-        <v>26000</v>
+        <v>32500</v>
       </c>
       <c r="E5" s="11" t="n">
-        <v>22000</v>
+        <v>27500</v>
       </c>
       <c r="F5" s="11">
         <f>D5+E5</f>
@@ -6509,10 +6509,10 @@
         </is>
       </c>
       <c r="D17" s="17" t="n">
-        <v>17490</v>
+        <v>18920</v>
       </c>
       <c r="E17" s="17" t="n">
-        <v>13860</v>
+        <v>15070</v>
       </c>
       <c r="F17" s="17">
         <f>D17+E17</f>
@@ -6551,10 +6551,10 @@
         </is>
       </c>
       <c r="D18" s="11" t="n">
-        <v>18365</v>
+        <v>19866</v>
       </c>
       <c r="E18" s="11" t="n">
-        <v>14553</v>
+        <v>15824</v>
       </c>
       <c r="F18" s="11">
         <f>D18+E18</f>
@@ -6593,10 +6593,10 @@
         </is>
       </c>
       <c r="D19" s="17" t="n">
-        <v>19283</v>
+        <v>20859</v>
       </c>
       <c r="E19" s="17" t="n">
-        <v>15281</v>
+        <v>16615</v>
       </c>
       <c r="F19" s="17">
         <f>D19+E19</f>
@@ -6635,10 +6635,10 @@
         </is>
       </c>
       <c r="D20" s="11" t="n">
-        <v>20247</v>
+        <v>21902</v>
       </c>
       <c r="E20" s="11" t="n">
-        <v>16045</v>
+        <v>17445</v>
       </c>
       <c r="F20" s="11">
         <f>D20+E20</f>
@@ -6677,10 +6677,10 @@
         </is>
       </c>
       <c r="D21" s="17" t="n">
-        <v>21259</v>
+        <v>22997</v>
       </c>
       <c r="E21" s="17" t="n">
-        <v>16847</v>
+        <v>18318</v>
       </c>
       <c r="F21" s="17">
         <f>D21+E21</f>

</xml_diff>